<commit_message>
Update workflow, sample data, docs and add demo screenshots
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -179,12 +179,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$7:$A$16</f>
+              <f>'Dashboard'!$A$7:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$7:$B$16</f>
+              <f>'Dashboard'!$B$7:$B$12</f>
             </numRef>
           </val>
         </ser>
@@ -291,12 +291,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$D$7:$D$16</f>
+              <f>'Dashboard'!$D$7:$D$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$7:$E$16</f>
+              <f>'Dashboard'!$E$7:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -710,8 +710,8 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -765,17 +765,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gwenborough</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Romaguera-Crona</t>
+          <t>GlobalTech</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -797,17 +797,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wisokyburgh</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Deckow-Crist</t>
+          <t>GlobalTech</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -829,17 +829,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>McKenziehaven</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Romaguera-Jacobson</t>
+          <t>DataSystems</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -861,17 +861,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>South Elvis</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Robel-Corkery</t>
+          <t>DataSystems</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -893,17 +893,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Roscoeview</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Keebler LLC</t>
+          <t>CloudBase</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -925,17 +925,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>South Christy</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Considine-Lockman</t>
+          <t>CloudBase</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -957,12 +957,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Howemouth</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Johns Group</t>
+          <t>NovaSoft</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -989,17 +989,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Aliyaview</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Abernathy Group</t>
+          <t>NovaSoft</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1021,17 +1021,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bartholomebury</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Yost and Sons</t>
+          <t>GlobalTech</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lebsackbury</t>
+          <t>Sydney</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hoeger LLC</t>
+          <t>DataSystems</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1078,13 +1078,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="2" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1144,7 +1144,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aliyaview</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1152,53 +1152,53 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Abernathy Group</t>
+          <t>CloudBase</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bartholomebury</t>
+          <t>London</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Considine-Lockman</t>
+          <t>DataSystems</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gwenborough</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Deckow-Crist</t>
+          <t>GlobalTech</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Howemouth</t>
+          <t>Sydney</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1206,119 +1206,31 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hoeger LLC</t>
+          <t>NovaSoft</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lebsackbury</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Johns Group</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>McKenziehaven</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>1</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Keebler LLC</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Roscoeview</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Robel-Corkery</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>South Christy</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Romaguera-Crona</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>South Elvis</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Romaguera-Jacobson</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Wisokyburgh</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Yost and Sons</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>